<commit_message>
Add mine warfare ship type to templates, regression, predictions and reports
</commit_message>
<xml_diff>
--- a/downloads/실적함_입력양식.xlsx
+++ b/downloads/실적함_입력양식.xlsx
@@ -476,8 +476,8 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B10000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="함종 확인" error="구축함, 호위함, 고속함, 지원함, 상륙함 중 선택하세요." type="list">
-      <formula1>"구축함,호위함,고속함,지원함,상륙함"</formula1>
+    <dataValidation sqref="B2:B10000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="함종 확인" error="구축함, 호위함, 고속함, 지원함, 상륙함, 기뢰전함 중 선택하세요." type="list">
+      <formula1>"구축함,호위함,고속함,지원함,상륙함,기뢰전함"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Remove support ship category and select largest observed type as reference
</commit_message>
<xml_diff>
--- a/downloads/실적함_입력양식.xlsx
+++ b/downloads/실적함_입력양식.xlsx
@@ -476,8 +476,8 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B10000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="함종 확인" error="구축함, 호위함, 고속함, 지원함, 상륙함, 기뢰전함 중 선택하세요." type="list">
-      <formula1>"구축함,호위함,고속함,지원함,상륙함,기뢰전함"</formula1>
+    <dataValidation sqref="B2:B10000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="함종 확인" error="구축함, 호위함, 고속함, 상륙함, 기뢰전함 중 선택하세요." type="list">
+      <formula1>"구축함,호위함,고속함,상륙함,기뢰전함"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>